<commit_message>
chore: 更新 pacenote_view.xlsx 文件
</commit_message>
<xml_diff>
--- a/pacenote_view.xlsx
+++ b/pacenote_view.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\devfiles\auto_media_pack_acg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B163406-D167-444C-AB17-495FC344A8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C9DB99B-399B-4251-8777-DF07A084D7D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="144" yWindow="1296" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2894,9 +2894,6 @@
     <t>start_stage,system_start_stage</t>
   </si>
   <si>
-    <t>比赛开始骚话</t>
-  </si>
-  <si>
     <t>steep</t>
   </si>
   <si>
@@ -3513,13 +3510,17 @@
   </si>
   <si>
     <t>手杀</t>
+  </si>
+  <si>
+    <t>比赛开始</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3530,6 +3531,14 @@
     <font>
       <sz val="9"/>
       <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -3554,9 +3563,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -5858,7 +5868,7 @@
         <v>285</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="E85" s="1" t="s">
         <v>286</v>
@@ -6295,7 +6305,7 @@
         <v>345</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="E104" s="1" t="s">
         <v>286</v>
@@ -7514,7 +7524,7 @@
         <v>516</v>
       </c>
       <c r="D157" s="1" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="E157" s="1" t="s">
         <v>286</v>
@@ -10503,8 +10513,8 @@
       <c r="C287" s="1" t="s">
         <v>947</v>
       </c>
-      <c r="D287" s="1" t="s">
-        <v>948</v>
+      <c r="D287" s="2" t="s">
+        <v>1154</v>
       </c>
       <c r="E287" s="1" t="s">
         <v>323</v>
@@ -10521,13 +10531,13 @@
         <v>206</v>
       </c>
       <c r="B288" s="1" t="s">
+        <v>948</v>
+      </c>
+      <c r="C288" s="1" t="s">
         <v>949</v>
       </c>
-      <c r="C288" s="1" t="s">
+      <c r="D288" s="1" t="s">
         <v>950</v>
-      </c>
-      <c r="D288" s="1" t="s">
-        <v>951</v>
       </c>
       <c r="E288" s="1" t="s">
         <v>245</v>
@@ -10544,13 +10554,13 @@
         <v>207</v>
       </c>
       <c r="B289" s="1" t="s">
+        <v>951</v>
+      </c>
+      <c r="C289" s="1" t="s">
         <v>952</v>
       </c>
-      <c r="C289" s="1" t="s">
+      <c r="D289" s="1" t="s">
         <v>953</v>
-      </c>
-      <c r="D289" s="1" t="s">
-        <v>954</v>
       </c>
       <c r="E289" s="1" t="s">
         <v>249</v>
@@ -10559,7 +10569,7 @@
         <v>209</v>
       </c>
       <c r="G289" s="1" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
     </row>
     <row r="290" spans="1:7" x14ac:dyDescent="0.25">
@@ -10567,13 +10577,13 @@
         <v>208</v>
       </c>
       <c r="B290" s="1" t="s">
+        <v>955</v>
+      </c>
+      <c r="C290" s="1" t="s">
         <v>956</v>
       </c>
-      <c r="C290" s="1" t="s">
-        <v>957</v>
-      </c>
       <c r="D290" s="1" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="E290" s="1" t="s">
         <v>249</v>
@@ -10582,7 +10592,7 @@
         <v>209</v>
       </c>
       <c r="G290" s="1" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
     </row>
     <row r="291" spans="1:7" x14ac:dyDescent="0.25">
@@ -10590,13 +10600,13 @@
         <v>209</v>
       </c>
       <c r="B291" s="1" t="s">
+        <v>957</v>
+      </c>
+      <c r="C291" s="1" t="s">
         <v>958</v>
       </c>
-      <c r="C291" s="1" t="s">
-        <v>959</v>
-      </c>
       <c r="D291" s="1" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="E291" s="1" t="s">
         <v>249</v>
@@ -10605,7 +10615,7 @@
         <v>209</v>
       </c>
       <c r="G291" s="1" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
     </row>
     <row r="292" spans="1:7" x14ac:dyDescent="0.25">
@@ -10613,13 +10623,13 @@
         <v>210</v>
       </c>
       <c r="B292" s="1" t="s">
+        <v>959</v>
+      </c>
+      <c r="C292" s="1" t="s">
         <v>960</v>
       </c>
-      <c r="C292" s="1" t="s">
+      <c r="D292" s="1" t="s">
         <v>961</v>
-      </c>
-      <c r="D292" s="1" t="s">
-        <v>962</v>
       </c>
       <c r="E292" s="1" t="s">
         <v>286</v>
@@ -10636,13 +10646,13 @@
         <v>211</v>
       </c>
       <c r="B293" s="1" t="s">
+        <v>962</v>
+      </c>
+      <c r="C293" s="1" t="s">
         <v>963</v>
       </c>
-      <c r="C293" s="1" t="s">
+      <c r="D293" s="1" t="s">
         <v>964</v>
-      </c>
-      <c r="D293" s="1" t="s">
-        <v>965</v>
       </c>
       <c r="E293" s="1" t="s">
         <v>286</v>
@@ -10659,10 +10669,10 @@
         <v>212</v>
       </c>
       <c r="B294" s="1" t="s">
+        <v>965</v>
+      </c>
+      <c r="C294" s="1" t="s">
         <v>966</v>
-      </c>
-      <c r="C294" s="1" t="s">
-        <v>967</v>
       </c>
       <c r="D294" s="1" t="s">
         <v>937</v>
@@ -10682,13 +10692,13 @@
         <v>213</v>
       </c>
       <c r="B295" s="1" t="s">
+        <v>967</v>
+      </c>
+      <c r="C295" s="1" t="s">
         <v>968</v>
       </c>
-      <c r="C295" s="1" t="s">
+      <c r="D295" s="1" t="s">
         <v>969</v>
-      </c>
-      <c r="D295" s="1" t="s">
-        <v>970</v>
       </c>
       <c r="E295" s="1" t="s">
         <v>201</v>
@@ -10705,13 +10715,13 @@
         <v>214</v>
       </c>
       <c r="B296" s="1" t="s">
+        <v>970</v>
+      </c>
+      <c r="C296" s="1" t="s">
         <v>971</v>
       </c>
-      <c r="C296" s="1" t="s">
+      <c r="D296" s="1" t="s">
         <v>972</v>
-      </c>
-      <c r="D296" s="1" t="s">
-        <v>973</v>
       </c>
       <c r="E296" s="1" t="s">
         <v>286</v>
@@ -10728,13 +10738,13 @@
         <v>215</v>
       </c>
       <c r="B297" s="1" t="s">
+        <v>973</v>
+      </c>
+      <c r="C297" s="1" t="s">
         <v>974</v>
       </c>
-      <c r="C297" s="1" t="s">
+      <c r="D297" s="1" t="s">
         <v>975</v>
-      </c>
-      <c r="D297" s="1" t="s">
-        <v>976</v>
       </c>
       <c r="E297" s="1" t="s">
         <v>208</v>
@@ -10751,13 +10761,13 @@
         <v>216</v>
       </c>
       <c r="B298" s="1" t="s">
+        <v>976</v>
+      </c>
+      <c r="C298" s="1" t="s">
         <v>977</v>
       </c>
-      <c r="C298" s="1" t="s">
+      <c r="D298" s="1" t="s">
         <v>978</v>
-      </c>
-      <c r="D298" s="1" t="s">
-        <v>979</v>
       </c>
       <c r="E298" s="1" t="s">
         <v>319</v>
@@ -10774,13 +10784,13 @@
         <v>217</v>
       </c>
       <c r="B299" s="1" t="s">
+        <v>979</v>
+      </c>
+      <c r="C299" s="1" t="s">
         <v>980</v>
       </c>
-      <c r="C299" s="1" t="s">
+      <c r="D299" s="1" t="s">
         <v>981</v>
-      </c>
-      <c r="D299" s="1" t="s">
-        <v>982</v>
       </c>
       <c r="E299" s="1" t="s">
         <v>201</v>
@@ -10797,13 +10807,13 @@
         <v>218</v>
       </c>
       <c r="B300" s="1" t="s">
+        <v>982</v>
+      </c>
+      <c r="C300" s="1" t="s">
         <v>983</v>
       </c>
-      <c r="C300" s="1" t="s">
+      <c r="D300" s="1" t="s">
         <v>984</v>
-      </c>
-      <c r="D300" s="1" t="s">
-        <v>985</v>
       </c>
       <c r="E300" s="1" t="s">
         <v>201</v>
@@ -10820,13 +10830,13 @@
         <v>334</v>
       </c>
       <c r="B301" s="1" t="s">
+        <v>985</v>
+      </c>
+      <c r="C301" s="1" t="s">
         <v>986</v>
       </c>
-      <c r="C301" s="1" t="s">
+      <c r="D301" s="1" t="s">
         <v>987</v>
-      </c>
-      <c r="D301" s="1" t="s">
-        <v>988</v>
       </c>
       <c r="E301" s="1" t="s">
         <v>208</v>
@@ -10835,7 +10845,7 @@
         <v>209</v>
       </c>
       <c r="G301" s="1" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
     </row>
     <row r="302" spans="1:7" x14ac:dyDescent="0.25">
@@ -10843,13 +10853,13 @@
         <v>219</v>
       </c>
       <c r="B302" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C302" s="1" t="s">
         <v>990</v>
       </c>
-      <c r="C302" s="1" t="s">
+      <c r="D302" s="1" t="s">
         <v>991</v>
-      </c>
-      <c r="D302" s="1" t="s">
-        <v>992</v>
       </c>
       <c r="E302" s="1" t="s">
         <v>249</v>
@@ -10858,7 +10868,7 @@
         <v>209</v>
       </c>
       <c r="G302" s="1" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
     </row>
     <row r="303" spans="1:7" x14ac:dyDescent="0.25">
@@ -10866,13 +10876,13 @@
         <v>220</v>
       </c>
       <c r="B303" s="1" t="s">
+        <v>993</v>
+      </c>
+      <c r="C303" s="1" t="s">
         <v>994</v>
       </c>
-      <c r="C303" s="1" t="s">
+      <c r="D303" s="1" t="s">
         <v>995</v>
-      </c>
-      <c r="D303" s="1" t="s">
-        <v>996</v>
       </c>
       <c r="E303" s="1" t="s">
         <v>208</v>
@@ -10881,7 +10891,7 @@
         <v>209</v>
       </c>
       <c r="G303" s="1" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
     </row>
     <row r="304" spans="1:7" x14ac:dyDescent="0.25">
@@ -10889,13 +10899,13 @@
         <v>221</v>
       </c>
       <c r="B304" s="1" t="s">
+        <v>997</v>
+      </c>
+      <c r="C304" s="1" t="s">
         <v>998</v>
       </c>
-      <c r="C304" s="1" t="s">
+      <c r="D304" s="1" t="s">
         <v>999</v>
-      </c>
-      <c r="D304" s="1" t="s">
-        <v>1000</v>
       </c>
       <c r="E304" s="1" t="s">
         <v>249</v>
@@ -10904,7 +10914,7 @@
         <v>209</v>
       </c>
       <c r="G304" s="1" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="305" spans="1:7" x14ac:dyDescent="0.25">
@@ -10912,13 +10922,13 @@
         <v>222</v>
       </c>
       <c r="B305" s="1" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C305" s="1" t="s">
         <v>1002</v>
       </c>
-      <c r="C305" s="1" t="s">
+      <c r="D305" s="1" t="s">
         <v>1003</v>
-      </c>
-      <c r="D305" s="1" t="s">
-        <v>1004</v>
       </c>
       <c r="E305" s="1" t="s">
         <v>208</v>
@@ -10927,7 +10937,7 @@
         <v>209</v>
       </c>
       <c r="G305" s="1" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="306" spans="1:7" x14ac:dyDescent="0.25">
@@ -10935,13 +10945,13 @@
         <v>330</v>
       </c>
       <c r="B306" s="1" t="s">
+        <v>1005</v>
+      </c>
+      <c r="C306" s="1" t="s">
         <v>1006</v>
       </c>
-      <c r="C306" s="1" t="s">
+      <c r="D306" s="1" t="s">
         <v>1007</v>
-      </c>
-      <c r="D306" s="1" t="s">
-        <v>1008</v>
       </c>
       <c r="E306" s="1" t="s">
         <v>249</v>
@@ -10950,7 +10960,7 @@
         <v>209</v>
       </c>
       <c r="G306" s="1" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="307" spans="1:7" x14ac:dyDescent="0.25">
@@ -10958,13 +10968,13 @@
         <v>223</v>
       </c>
       <c r="B307" s="1" t="s">
+        <v>1009</v>
+      </c>
+      <c r="C307" s="1" t="s">
         <v>1010</v>
       </c>
-      <c r="C307" s="1" t="s">
+      <c r="D307" s="1" t="s">
         <v>1011</v>
-      </c>
-      <c r="D307" s="1" t="s">
-        <v>1012</v>
       </c>
       <c r="E307" s="1" t="s">
         <v>208</v>
@@ -10973,7 +10983,7 @@
         <v>209</v>
       </c>
       <c r="G307" s="1" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="308" spans="1:7" x14ac:dyDescent="0.25">
@@ -10981,13 +10991,13 @@
         <v>224</v>
       </c>
       <c r="B308" s="1" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C308" s="1" t="s">
         <v>1014</v>
       </c>
-      <c r="C308" s="1" t="s">
+      <c r="D308" s="1" t="s">
         <v>1015</v>
-      </c>
-      <c r="D308" s="1" t="s">
-        <v>1016</v>
       </c>
       <c r="E308" s="1" t="s">
         <v>208</v>
@@ -10996,7 +11006,7 @@
         <v>209</v>
       </c>
       <c r="G308" s="1" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="309" spans="1:7" x14ac:dyDescent="0.25">
@@ -11004,13 +11014,13 @@
         <v>225</v>
       </c>
       <c r="B309" s="1" t="s">
+        <v>1017</v>
+      </c>
+      <c r="C309" s="1" t="s">
         <v>1018</v>
       </c>
-      <c r="C309" s="1" t="s">
+      <c r="D309" s="1" t="s">
         <v>1019</v>
-      </c>
-      <c r="D309" s="1" t="s">
-        <v>1020</v>
       </c>
       <c r="E309" s="1" t="s">
         <v>249</v>
@@ -11019,7 +11029,7 @@
         <v>209</v>
       </c>
       <c r="G309" s="1" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="310" spans="1:7" x14ac:dyDescent="0.25">
@@ -11027,13 +11037,13 @@
         <v>226</v>
       </c>
       <c r="B310" s="1" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C310" s="1" t="s">
         <v>1022</v>
       </c>
-      <c r="C310" s="1" t="s">
+      <c r="D310" s="1" t="s">
         <v>1023</v>
-      </c>
-      <c r="D310" s="1" t="s">
-        <v>1024</v>
       </c>
       <c r="E310" s="1" t="s">
         <v>208</v>
@@ -11042,7 +11052,7 @@
         <v>209</v>
       </c>
       <c r="G310" s="1" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="311" spans="1:7" x14ac:dyDescent="0.25">
@@ -11050,13 +11060,13 @@
         <v>227</v>
       </c>
       <c r="B311" s="1" t="s">
+        <v>1025</v>
+      </c>
+      <c r="C311" s="1" t="s">
         <v>1026</v>
       </c>
-      <c r="C311" s="1" t="s">
+      <c r="D311" s="1" t="s">
         <v>1027</v>
-      </c>
-      <c r="D311" s="1" t="s">
-        <v>1028</v>
       </c>
       <c r="E311" s="1" t="s">
         <v>249</v>
@@ -11065,7 +11075,7 @@
         <v>209</v>
       </c>
       <c r="G311" s="1" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="312" spans="1:7" x14ac:dyDescent="0.25">
@@ -11073,13 +11083,13 @@
         <v>228</v>
       </c>
       <c r="B312" s="1" t="s">
+        <v>1029</v>
+      </c>
+      <c r="C312" s="1" t="s">
         <v>1030</v>
       </c>
-      <c r="C312" s="1" t="s">
+      <c r="D312" s="1" t="s">
         <v>1031</v>
-      </c>
-      <c r="D312" s="1" t="s">
-        <v>1032</v>
       </c>
       <c r="E312" s="1" t="s">
         <v>437</v>
@@ -11096,13 +11106,13 @@
         <v>229</v>
       </c>
       <c r="B313" s="1" t="s">
+        <v>1032</v>
+      </c>
+      <c r="C313" s="1" t="s">
         <v>1033</v>
       </c>
-      <c r="C313" s="1" t="s">
+      <c r="D313" s="1" t="s">
         <v>1034</v>
-      </c>
-      <c r="D313" s="1" t="s">
-        <v>1035</v>
       </c>
       <c r="E313" s="1" t="s">
         <v>437</v>
@@ -11111,7 +11121,7 @@
         <v>209</v>
       </c>
       <c r="G313" s="1" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="314" spans="1:7" x14ac:dyDescent="0.25">
@@ -11119,13 +11129,13 @@
         <v>317</v>
       </c>
       <c r="B314" s="1" t="s">
+        <v>1036</v>
+      </c>
+      <c r="C314" s="1" t="s">
         <v>1037</v>
       </c>
-      <c r="C314" s="1" t="s">
+      <c r="D314" s="1" t="s">
         <v>1038</v>
-      </c>
-      <c r="D314" s="1" t="s">
-        <v>1039</v>
       </c>
       <c r="E314" s="1" t="s">
         <v>50</v>
@@ -11142,13 +11152,13 @@
         <v>230</v>
       </c>
       <c r="B315" s="1" t="s">
+        <v>1039</v>
+      </c>
+      <c r="C315" s="1" t="s">
         <v>1040</v>
       </c>
-      <c r="C315" s="1" t="s">
+      <c r="D315" s="1" t="s">
         <v>1041</v>
-      </c>
-      <c r="D315" s="1" t="s">
-        <v>1042</v>
       </c>
       <c r="E315" s="1" t="s">
         <v>50</v>
@@ -11157,7 +11167,7 @@
         <v>209</v>
       </c>
       <c r="G315" s="1" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="316" spans="1:7" x14ac:dyDescent="0.25">
@@ -11165,13 +11175,13 @@
         <v>231</v>
       </c>
       <c r="B316" s="1" t="s">
+        <v>1043</v>
+      </c>
+      <c r="C316" s="1" t="s">
         <v>1044</v>
       </c>
-      <c r="C316" s="1" t="s">
+      <c r="D316" s="1" t="s">
         <v>1045</v>
-      </c>
-      <c r="D316" s="1" t="s">
-        <v>1046</v>
       </c>
       <c r="E316" s="1" t="s">
         <v>50</v>
@@ -11180,7 +11190,7 @@
         <v>209</v>
       </c>
       <c r="G316" s="1" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="317" spans="1:7" x14ac:dyDescent="0.25">
@@ -11188,13 +11198,13 @@
         <v>232</v>
       </c>
       <c r="B317" s="1" t="s">
+        <v>1047</v>
+      </c>
+      <c r="C317" s="1" t="s">
         <v>1048</v>
       </c>
-      <c r="C317" s="1" t="s">
+      <c r="D317" s="1" t="s">
         <v>1049</v>
-      </c>
-      <c r="D317" s="1" t="s">
-        <v>1050</v>
       </c>
       <c r="E317" s="1" t="s">
         <v>50</v>
@@ -11203,7 +11213,7 @@
         <v>209</v>
       </c>
       <c r="G317" s="1" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="318" spans="1:7" x14ac:dyDescent="0.25">
@@ -11211,13 +11221,13 @@
         <v>233</v>
       </c>
       <c r="B318" s="1" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C318" s="1" t="s">
         <v>1052</v>
       </c>
-      <c r="C318" s="1" t="s">
+      <c r="D318" s="1" t="s">
         <v>1053</v>
-      </c>
-      <c r="D318" s="1" t="s">
-        <v>1054</v>
       </c>
       <c r="E318" s="1" t="s">
         <v>50</v>
@@ -11226,7 +11236,7 @@
         <v>209</v>
       </c>
       <c r="G318" s="1" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="319" spans="1:7" x14ac:dyDescent="0.25">
@@ -11234,13 +11244,13 @@
         <v>234</v>
       </c>
       <c r="B319" s="1" t="s">
+        <v>1055</v>
+      </c>
+      <c r="C319" s="1" t="s">
         <v>1056</v>
       </c>
-      <c r="C319" s="1" t="s">
+      <c r="D319" s="1" t="s">
         <v>1057</v>
-      </c>
-      <c r="D319" s="1" t="s">
-        <v>1058</v>
       </c>
       <c r="E319" s="1" t="s">
         <v>50</v>
@@ -11249,7 +11259,7 @@
         <v>209</v>
       </c>
       <c r="G319" s="1" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="320" spans="1:7" x14ac:dyDescent="0.25">
@@ -11257,13 +11267,13 @@
         <v>323</v>
       </c>
       <c r="B320" s="1" t="s">
+        <v>1059</v>
+      </c>
+      <c r="C320" s="1" t="s">
         <v>1060</v>
       </c>
-      <c r="C320" s="1" t="s">
+      <c r="D320" s="1" t="s">
         <v>1061</v>
-      </c>
-      <c r="D320" s="1" t="s">
-        <v>1062</v>
       </c>
       <c r="E320" s="1" t="s">
         <v>50</v>
@@ -11272,7 +11282,7 @@
         <v>209</v>
       </c>
       <c r="G320" s="1" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="321" spans="1:7" x14ac:dyDescent="0.25">
@@ -11280,13 +11290,13 @@
         <v>309</v>
       </c>
       <c r="B321" s="1" t="s">
+        <v>1063</v>
+      </c>
+      <c r="C321" s="1" t="s">
         <v>1064</v>
       </c>
-      <c r="C321" s="1" t="s">
+      <c r="D321" s="1" t="s">
         <v>1065</v>
-      </c>
-      <c r="D321" s="1" t="s">
-        <v>1066</v>
       </c>
       <c r="E321" s="1" t="s">
         <v>50</v>
@@ -11295,7 +11305,7 @@
         <v>209</v>
       </c>
       <c r="G321" s="1" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="322" spans="1:7" x14ac:dyDescent="0.25">
@@ -11303,13 +11313,13 @@
         <v>235</v>
       </c>
       <c r="B322" s="1" t="s">
+        <v>1067</v>
+      </c>
+      <c r="C322" s="1" t="s">
         <v>1068</v>
       </c>
-      <c r="C322" s="1" t="s">
+      <c r="D322" s="1" t="s">
         <v>1069</v>
-      </c>
-      <c r="D322" s="1" t="s">
-        <v>1070</v>
       </c>
       <c r="E322" s="1" t="s">
         <v>50</v>
@@ -11318,7 +11328,7 @@
         <v>209</v>
       </c>
       <c r="G322" s="1" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="323" spans="1:7" x14ac:dyDescent="0.25">
@@ -11326,13 +11336,13 @@
         <v>325</v>
       </c>
       <c r="B323" s="1" t="s">
+        <v>1071</v>
+      </c>
+      <c r="C323" s="1" t="s">
         <v>1072</v>
       </c>
-      <c r="C323" s="1" t="s">
+      <c r="D323" s="1" t="s">
         <v>1073</v>
-      </c>
-      <c r="D323" s="1" t="s">
-        <v>1074</v>
       </c>
       <c r="E323" s="1" t="s">
         <v>50</v>
@@ -11341,7 +11351,7 @@
         <v>209</v>
       </c>
       <c r="G323" s="1" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="324" spans="1:7" x14ac:dyDescent="0.25">
@@ -11349,13 +11359,13 @@
         <v>236</v>
       </c>
       <c r="B324" s="1" t="s">
+        <v>1075</v>
+      </c>
+      <c r="C324" s="1" t="s">
         <v>1076</v>
       </c>
-      <c r="C324" s="1" t="s">
+      <c r="D324" s="1" t="s">
         <v>1077</v>
-      </c>
-      <c r="D324" s="1" t="s">
-        <v>1078</v>
       </c>
       <c r="E324" s="1" t="s">
         <v>50</v>
@@ -11364,7 +11374,7 @@
         <v>209</v>
       </c>
       <c r="G324" s="1" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="325" spans="1:7" x14ac:dyDescent="0.25">
@@ -11372,13 +11382,13 @@
         <v>237</v>
       </c>
       <c r="B325" s="1" t="s">
+        <v>1079</v>
+      </c>
+      <c r="C325" s="1" t="s">
         <v>1080</v>
       </c>
-      <c r="C325" s="1" t="s">
+      <c r="D325" s="1" t="s">
         <v>1081</v>
-      </c>
-      <c r="D325" s="1" t="s">
-        <v>1082</v>
       </c>
       <c r="E325" s="1" t="s">
         <v>208</v>
@@ -11395,13 +11405,13 @@
         <v>238</v>
       </c>
       <c r="B326" s="1" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C326" s="1" t="s">
         <v>1083</v>
       </c>
-      <c r="C326" s="1" t="s">
+      <c r="D326" s="1" t="s">
         <v>1084</v>
-      </c>
-      <c r="D326" s="1" t="s">
-        <v>1085</v>
       </c>
       <c r="E326" s="1" t="s">
         <v>208</v>
@@ -11410,7 +11420,7 @@
         <v>209</v>
       </c>
       <c r="G326" s="1" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="327" spans="1:7" x14ac:dyDescent="0.25">
@@ -11418,13 +11428,13 @@
         <v>239</v>
       </c>
       <c r="B327" s="1" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C327" s="1" t="s">
         <v>1087</v>
       </c>
-      <c r="C327" s="1" t="s">
+      <c r="D327" s="1" t="s">
         <v>1088</v>
-      </c>
-      <c r="D327" s="1" t="s">
-        <v>1089</v>
       </c>
       <c r="E327" s="1" t="s">
         <v>208</v>
@@ -11433,7 +11443,7 @@
         <v>209</v>
       </c>
       <c r="G327" s="1" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="328" spans="1:7" x14ac:dyDescent="0.25">
@@ -11441,13 +11451,13 @@
         <v>295</v>
       </c>
       <c r="B328" s="1" t="s">
+        <v>1090</v>
+      </c>
+      <c r="C328" s="1" t="s">
         <v>1091</v>
       </c>
-      <c r="C328" s="1" t="s">
+      <c r="D328" s="1" t="s">
         <v>1092</v>
-      </c>
-      <c r="D328" s="1" t="s">
-        <v>1093</v>
       </c>
       <c r="E328" s="1" t="s">
         <v>245</v>
@@ -11464,13 +11474,13 @@
         <v>240</v>
       </c>
       <c r="B329" s="1" t="s">
+        <v>1093</v>
+      </c>
+      <c r="C329" s="1" t="s">
         <v>1094</v>
       </c>
-      <c r="C329" s="1" t="s">
+      <c r="D329" s="1" t="s">
         <v>1095</v>
-      </c>
-      <c r="D329" s="1" t="s">
-        <v>1096</v>
       </c>
       <c r="E329" s="1" t="s">
         <v>290</v>
@@ -11479,7 +11489,7 @@
         <v>209</v>
       </c>
       <c r="G329" s="1" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="330" spans="1:7" x14ac:dyDescent="0.25">
@@ -11487,13 +11497,13 @@
         <v>241</v>
       </c>
       <c r="B330" s="1" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C330" s="1" t="s">
         <v>1098</v>
       </c>
-      <c r="C330" s="1" t="s">
+      <c r="D330" s="1" t="s">
         <v>1099</v>
-      </c>
-      <c r="D330" s="1" t="s">
-        <v>1100</v>
       </c>
       <c r="E330" s="1" t="s">
         <v>290</v>
@@ -11510,13 +11520,13 @@
         <v>242</v>
       </c>
       <c r="B331" s="1" t="s">
+        <v>1100</v>
+      </c>
+      <c r="C331" s="1" t="s">
         <v>1101</v>
       </c>
-      <c r="C331" s="1" t="s">
+      <c r="D331" s="1" t="s">
         <v>1102</v>
-      </c>
-      <c r="D331" s="1" t="s">
-        <v>1103</v>
       </c>
       <c r="E331" s="1" t="s">
         <v>249</v>
@@ -11533,13 +11543,13 @@
         <v>243</v>
       </c>
       <c r="B332" s="1" t="s">
+        <v>1103</v>
+      </c>
+      <c r="C332" s="1" t="s">
         <v>1104</v>
       </c>
-      <c r="C332" s="1" t="s">
+      <c r="D332" s="1" t="s">
         <v>1105</v>
-      </c>
-      <c r="D332" s="1" t="s">
-        <v>1106</v>
       </c>
       <c r="E332" s="1" t="s">
         <v>201</v>
@@ -11559,10 +11569,10 @@
         <v>575</v>
       </c>
       <c r="C333" s="1" t="s">
+        <v>1106</v>
+      </c>
+      <c r="D333" s="1" t="s">
         <v>1107</v>
-      </c>
-      <c r="D333" s="1" t="s">
-        <v>1108</v>
       </c>
       <c r="E333" s="1" t="s">
         <v>275</v>
@@ -11579,13 +11589,13 @@
         <v>26</v>
       </c>
       <c r="B334" s="1" t="s">
+        <v>1108</v>
+      </c>
+      <c r="C334" s="1" t="s">
         <v>1109</v>
       </c>
-      <c r="C334" s="1" t="s">
+      <c r="D334" s="1" t="s">
         <v>1110</v>
-      </c>
-      <c r="D334" s="1" t="s">
-        <v>1111</v>
       </c>
       <c r="E334" s="1" t="s">
         <v>50</v>
@@ -11602,13 +11612,13 @@
         <v>27</v>
       </c>
       <c r="B335" s="1" t="s">
+        <v>1111</v>
+      </c>
+      <c r="C335" s="1" t="s">
         <v>1112</v>
       </c>
-      <c r="C335" s="1" t="s">
+      <c r="D335" s="1" t="s">
         <v>1113</v>
-      </c>
-      <c r="D335" s="1" t="s">
-        <v>1114</v>
       </c>
       <c r="E335" s="1" t="s">
         <v>50</v>
@@ -11625,13 +11635,13 @@
         <v>245</v>
       </c>
       <c r="B336" s="1" t="s">
+        <v>1114</v>
+      </c>
+      <c r="C336" s="1" t="s">
         <v>1115</v>
       </c>
-      <c r="C336" s="1" t="s">
+      <c r="D336" s="1" t="s">
         <v>1116</v>
-      </c>
-      <c r="D336" s="1" t="s">
-        <v>1117</v>
       </c>
       <c r="E336" s="1" t="s">
         <v>208</v>
@@ -11648,13 +11658,13 @@
         <v>246</v>
       </c>
       <c r="B337" s="1" t="s">
+        <v>1117</v>
+      </c>
+      <c r="C337" s="1" t="s">
         <v>1118</v>
       </c>
-      <c r="C337" s="1" t="s">
+      <c r="D337" s="1" t="s">
         <v>1119</v>
-      </c>
-      <c r="D337" s="1" t="s">
-        <v>1120</v>
       </c>
       <c r="E337" s="1" t="s">
         <v>286</v>
@@ -11671,13 +11681,13 @@
         <v>247</v>
       </c>
       <c r="B338" s="1" t="s">
+        <v>1120</v>
+      </c>
+      <c r="C338" s="1" t="s">
         <v>1121</v>
       </c>
-      <c r="C338" s="1" t="s">
+      <c r="D338" s="1" t="s">
         <v>1122</v>
-      </c>
-      <c r="D338" s="1" t="s">
-        <v>1123</v>
       </c>
       <c r="E338" s="1" t="s">
         <v>290</v>
@@ -11694,13 +11704,13 @@
         <v>248</v>
       </c>
       <c r="B339" s="1" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C339" s="1" t="s">
         <v>1124</v>
       </c>
-      <c r="C339" s="1" t="s">
+      <c r="D339" s="1" t="s">
         <v>1125</v>
-      </c>
-      <c r="D339" s="1" t="s">
-        <v>1126</v>
       </c>
       <c r="E339" s="1" t="s">
         <v>201</v>
@@ -11717,13 +11727,13 @@
         <v>249</v>
       </c>
       <c r="B340" s="1" t="s">
+        <v>1126</v>
+      </c>
+      <c r="C340" s="1" t="s">
         <v>1127</v>
       </c>
-      <c r="C340" s="1" t="s">
+      <c r="D340" s="1" t="s">
         <v>1128</v>
-      </c>
-      <c r="D340" s="1" t="s">
-        <v>1129</v>
       </c>
       <c r="E340" s="1" t="s">
         <v>249</v>
@@ -11740,13 +11750,13 @@
         <v>250</v>
       </c>
       <c r="B341" s="1" t="s">
+        <v>1129</v>
+      </c>
+      <c r="C341" s="1" t="s">
         <v>1130</v>
       </c>
-      <c r="C341" s="1" t="s">
+      <c r="D341" s="1" t="s">
         <v>1131</v>
-      </c>
-      <c r="D341" s="1" t="s">
-        <v>1132</v>
       </c>
       <c r="E341" s="1" t="s">
         <v>245</v>
@@ -11763,13 +11773,13 @@
         <v>135</v>
       </c>
       <c r="B342" s="1" t="s">
+        <v>1132</v>
+      </c>
+      <c r="C342" s="1" t="s">
         <v>1133</v>
       </c>
-      <c r="C342" s="1" t="s">
+      <c r="D342" s="1" t="s">
         <v>1134</v>
-      </c>
-      <c r="D342" s="1" t="s">
-        <v>1135</v>
       </c>
       <c r="E342" s="1" t="s">
         <v>437</v>
@@ -11778,7 +11788,7 @@
         <v>173</v>
       </c>
       <c r="G342" s="1" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="343" spans="1:7" x14ac:dyDescent="0.25">
@@ -11786,13 +11796,13 @@
         <v>251</v>
       </c>
       <c r="B343" s="1" t="s">
+        <v>1136</v>
+      </c>
+      <c r="C343" s="1" t="s">
         <v>1137</v>
       </c>
-      <c r="C343" s="1" t="s">
+      <c r="D343" s="1" t="s">
         <v>1138</v>
-      </c>
-      <c r="D343" s="1" t="s">
-        <v>1139</v>
       </c>
       <c r="E343" s="1" t="s">
         <v>286</v>
@@ -11809,13 +11819,13 @@
         <v>252</v>
       </c>
       <c r="B344" s="1" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C344" s="1" t="s">
         <v>1140</v>
       </c>
-      <c r="C344" s="1" t="s">
+      <c r="D344" s="1" t="s">
         <v>1141</v>
-      </c>
-      <c r="D344" s="1" t="s">
-        <v>1142</v>
       </c>
       <c r="E344" s="1" t="s">
         <v>208</v>
@@ -11832,13 +11842,13 @@
         <v>253</v>
       </c>
       <c r="B345" s="1" t="s">
+        <v>1142</v>
+      </c>
+      <c r="C345" s="1" t="s">
         <v>1143</v>
       </c>
-      <c r="C345" s="1" t="s">
+      <c r="D345" s="1" t="s">
         <v>1144</v>
-      </c>
-      <c r="D345" s="1" t="s">
-        <v>1145</v>
       </c>
       <c r="E345" s="1" t="s">
         <v>208</v>
@@ -11847,7 +11857,7 @@
         <v>209</v>
       </c>
       <c r="G345" s="1" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="346" spans="1:7" x14ac:dyDescent="0.25">
@@ -11855,13 +11865,13 @@
         <v>254</v>
       </c>
       <c r="B346" s="1" t="s">
+        <v>1145</v>
+      </c>
+      <c r="C346" s="1" t="s">
         <v>1146</v>
       </c>
-      <c r="C346" s="1" t="s">
+      <c r="D346" s="1" t="s">
         <v>1147</v>
-      </c>
-      <c r="D346" s="1" t="s">
-        <v>1148</v>
       </c>
       <c r="E346" s="1" t="s">
         <v>208</v>
@@ -11870,7 +11880,7 @@
         <v>209</v>
       </c>
       <c r="G346" s="1" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="347" spans="1:7" x14ac:dyDescent="0.25">
@@ -11878,13 +11888,13 @@
         <v>256</v>
       </c>
       <c r="B347" s="1" t="s">
+        <v>1148</v>
+      </c>
+      <c r="C347" s="1" t="s">
         <v>1149</v>
       </c>
-      <c r="C347" s="1" t="s">
+      <c r="D347" s="1" t="s">
         <v>1150</v>
-      </c>
-      <c r="D347" s="1" t="s">
-        <v>1151</v>
       </c>
       <c r="E347" s="1" t="s">
         <v>275</v>

</xml_diff>